<commit_message>
added batch declaration summary viewing and adding
</commit_message>
<xml_diff>
--- a/template/file/Gcash-Claim-Template.xlsx
+++ b/template/file/Gcash-Claim-Template.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="65">
   <si>
     <t>CUSTOMER FIRST NAME</t>
   </si>
@@ -206,13 +206,19 @@
     <t>BL1743675278034</t>
   </si>
   <si>
-    <t>TOTAL GINSURE BUY LOAD PROTECT PREMIUM</t>
-  </si>
-  <si>
-    <t>TOTAL GINSURE BUY LOAD PROTECT PREMIUM W TAXES</t>
-  </si>
-  <si>
-    <t>TOTAL GCASH SERVICE FEE</t>
+    <t>Christian</t>
+  </si>
+  <si>
+    <t>Carl</t>
+  </si>
+  <si>
+    <t>Jhustin</t>
+  </si>
+  <si>
+    <t>BATCH NUMBER</t>
+  </si>
+  <si>
+    <t>batch 200</t>
   </si>
 </sst>
 </file>
@@ -532,10 +538,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -584,10 +608,13 @@
       <c r="P1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -634,10 +661,13 @@
       <c r="P2" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
@@ -684,8 +714,11 @@
       <c r="P3" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -734,10 +767,13 @@
       <c r="P4" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
         <v>26</v>
@@ -784,10 +820,13 @@
       <c r="P5" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
@@ -834,8 +873,11 @@
       <c r="P6" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -884,8 +926,11 @@
       <c r="P7" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -934,8 +979,11 @@
       <c r="P8" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -984,8 +1032,11 @@
       <c r="P9" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1034,8 +1085,11 @@
       <c r="P10" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -1084,8 +1138,11 @@
       <c r="P11" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -1134,8 +1191,11 @@
       <c r="P12" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>38</v>
       </c>
@@ -1184,8 +1244,11 @@
       <c r="P13" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -1234,8 +1297,11 @@
       <c r="P14" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -1284,8 +1350,11 @@
       <c r="P15" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q15" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>52</v>
       </c>
@@ -1334,8 +1403,11 @@
       <c r="P16" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -1384,8 +1456,11 @@
       <c r="P17" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>46</v>
       </c>
@@ -1434,8 +1509,11 @@
       <c r="P18" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>52</v>
       </c>
@@ -1484,29 +1562,8 @@
       <c r="P19" s="2">
         <v>45753</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>60</v>
-      </c>
-      <c r="B21">
-        <v>405.09</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>61</v>
-      </c>
-      <c r="B22">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B23">
-        <v>147.86000000000001</v>
+      <c r="Q19" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>